<commit_message>
Label Cash timing units
</commit_message>
<xml_diff>
--- a/EOA_12_Month_Cash_Forecast.xlsx
+++ b/EOA_12_Month_Cash_Forecast.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12-Month Cash Forecast" sheetId="1" r:id="R7413ea5542d64610"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12-Month Cash Forecast" sheetId="1" r:id="Rfd18c3cb44c84b60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6346,7 +6346,7 @@
     </x:row>
     <x:row r="49" ht="22" customHeight="1">
       <x:c r="A49" s="118" t="str">
-        <x:v>Marketing timing</x:v>
+        <x:v>Marketing timing (months)</x:v>
       </x:c>
       <x:c r="B49" s="152" t="str">
         <x:f>IF(B7="","",B7)</x:f>
@@ -6483,7 +6483,7 @@
     </x:row>
     <x:row r="50" ht="22" customHeight="1">
       <x:c r="A50" s="118" t="str">
-        <x:v>Sales timing</x:v>
+        <x:v>Sales timing (months)</x:v>
       </x:c>
       <x:c r="B50" s="152" t="str">
         <x:f>IF(B12="","",B12)</x:f>
@@ -6622,7 +6622,7 @@
     </x:row>
     <x:row r="51" ht="22" customHeight="1">
       <x:c r="A51" s="118" t="str">
-        <x:v>Delivery timing</x:v>
+        <x:v>Delivery timing (months)</x:v>
       </x:c>
       <x:c r="B51" s="152" t="str">
         <x:f>IF(B19="","",B19)</x:f>
@@ -6761,7 +6761,7 @@
     </x:row>
     <x:row r="52" ht="22" customHeight="1">
       <x:c r="A52" s="118" t="str">
-        <x:v>Collection timing</x:v>
+        <x:v>Collection timing (months)</x:v>
       </x:c>
       <x:c r="B52" s="152" t="str">
         <x:f>IF(B31="","",B31)</x:f>

</xml_diff>